<commit_message>
added abelization and graphs added boltzman plots, temperature and atomic density before great refactor
</commit_message>
<xml_diff>
--- a/results/5153_gauss.xlsx
+++ b/results/5153_gauss.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,99 +413,87 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Radius</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>5153</t>
-        </is>
+      <c r="A1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B1" t="n">
+        <v>11.88051200089198</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0</v>
+        <v>0.341</v>
       </c>
       <c r="B2" t="n">
-        <v>752.2419962072357</v>
+        <v>11.77926875903428</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.186</v>
+        <v>0.6819999999999999</v>
       </c>
       <c r="B3" t="n">
-        <v>731.3760688007802</v>
+        <v>10.50238712185229</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.372</v>
+        <v>1.023</v>
       </c>
       <c r="B4" t="n">
-        <v>675.3977281679256</v>
+        <v>8.673001450666185</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.5735</v>
+        <v>1.364</v>
       </c>
       <c r="B5" t="n">
-        <v>578.5486041075668</v>
+        <v>6.666560902709706</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.7595</v>
+        <v>1.705</v>
       </c>
       <c r="B6" t="n">
-        <v>459.9434794804209</v>
+        <v>4.520743902844142</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.961</v>
+        <v>2.046</v>
       </c>
       <c r="B7" t="n">
-        <v>317.9747736018069</v>
+        <v>2.814522333000653</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1.147</v>
+        <v>2.387</v>
       </c>
       <c r="B8" t="n">
-        <v>191.8758918009861</v>
+        <v>1.522910362301926</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1.3485</v>
+        <v>2.728</v>
       </c>
       <c r="B9" t="n">
-        <v>86.09877134956666</v>
+        <v>0.7119160833722958</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1.5345</v>
+        <v>3.069</v>
       </c>
       <c r="B10" t="n">
-        <v>29.40105610787364</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>1.736</v>
-      </c>
-      <c r="B11" t="n">
-        <v>3.751309531058398</v>
+        <v>0.3117012869967862</v>
       </c>
     </row>
   </sheetData>

</xml_diff>